<commit_message>
Ajoute les questions refugie/handicap/stage au formulaire Kobo suivi
Nouvelles questions dans module_suivi (formulaire "suivi et satisfaction") :
- refugie + pays d'origine, handicap + type de handicap : mettent a jour la
  fiche du beneficiaire a chaque contact si renseignees (sans ecraser une
  valeur deja connue quand la question est laissee vide).
- structure d'accueil, encadrant, date de fin de stage (si situation =
  stage) : alimentent desormais l'Insertion correspondante.

Deploie via la nouvelle commande maj_formulaire_suivi_kobo, qui insere ces
lignes directement dans le formulaire deja en production (meme mecanisme
PATCH content + PATCH deployment que publier_beneficiaires_kobo), sans
creer de nouveau projet Kobo ni toucher a la liste des 1928 beneficiaires
deja publiee. Sauvegarde automatique de la definition precedente dans
kobo_forms/sauvegardes/ (non versionne) avant modification.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kobo_forms/suivi_et_satisfaction.xlsx
+++ b/kobo_forms/suivi_et_satisfaction.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,7 +742,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>date_fin_formation</t>
+          <t>domaine_formation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -754,7 +754,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>instance('beneficiaires')/root/item[name=current()/../id_beneficiaire]/date_fin_formation</t>
+          <t>instance('beneficiaires')/root/item[name=current()/../id_beneficiaire]/domaine_formation</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>telephone</t>
+          <t>date_fin_formation</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -779,7 +779,7 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>instance('beneficiaires')/root/item[name=current()/../id_beneficiaire]/telephone</t>
+          <t>instance('beneficiaires')/root/item[name=current()/../id_beneficiaire]/date_fin_formation</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -792,7 +792,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>mois_ecoules</t>
+          <t>telephone</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -804,7 +804,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>if(regex(${date_fin_formation}, '^[0-9]{4}-[0-9]{2}-[0-9]{2}$'), int((today() - date(${date_fin_formation})) div 30.4), '')</t>
+          <t>instance('beneficiaires')/root/item[name=current()/../id_beneficiaire]/telephone</t>
         </is>
       </c>
       <c r="K15" t="inlineStr"/>
@@ -812,57 +812,54 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>recapitulatif</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Bénéficiaire : ${nom_prenom} — ${institution} — ${region}
-Fin de formation : ${date_fin_formation} — ${mois_ecoules} mois écoulés
-Téléphone : ${telephone}</t>
-        </is>
-      </c>
+          <t>mois_ecoules</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>${id_beneficiaire} != ''</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>if(regex(${date_fin_formation}, '^[0-9]{4}-[0-9]{2}-[0-9]{2}$'), int((today() - date(${date_fin_formation})) div 30.4), '')</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>select_one canaux</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>canal</t>
+          <t>recapitulatif</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Canal du contact</t>
+          <t>Bénéficiaire : ${nom_prenom} — ${institution} — ${region}
+Formation suivie : ${domaine_formation}
+Fin de formation : ${date_fin_formation} — ${mois_ecoules} mois écoulés
+Téléphone : ${telephone}</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>${id_beneficiaire} != ''</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -872,17 +869,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one canaux</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>date_contact</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Date du contact</t>
+          <t>Canal du contact</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -892,71 +889,67 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>La date du contact ne peut pas être dans le futur.</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>today()</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>selection</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>date_contact</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Date du contact</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>. &lt;= today()</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>La date du contact ne peut pas être dans le futur.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>today()</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>select_one issues_contact</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>issue_contact</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Issue du contact</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Enregistré même en cas d'échec : c'est ce qui donne le taux de joignabilité.</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>selection</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -967,26 +960,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one issues_contact</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>note_echec</t>
+          <t>issue_contact</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Contact non abouti. Le questionnaire s'arrête ici : enregistrez et envoyez la soumission telle quelle.</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>${issue_contact} != 'joint'</t>
-        </is>
-      </c>
+          <t>Issue du contact</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Enregistré même en cas d'échec : c'est ce qui donne le taux de joignabilité.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
@@ -996,24 +993,24 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>module_suivi</t>
+          <t>note_echec</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Module 1 – Suivi de la situation</t>
+          <t>Contact non abouti. Le questionnaire s'arrête ici : enregistrez et envoyez la soumission telle quelle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>selected(${issue_contact}, 'joint')</t>
+          <t>${issue_contact} != 'joint'</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1025,26 +1022,26 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>select_one vagues</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>vague</t>
+          <t>module_suivi</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Vague de suivi</t>
+          <t>Module 1 – Suivi de la situation</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>selected(${issue_contact}, 'joint')</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
@@ -1054,17 +1051,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>select_one situations</t>
+          <t>select_one vagues</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>situation</t>
+          <t>vague</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Quelle est votre situation aujourd'hui ?</t>
+          <t>Vague de suivi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1083,17 +1080,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>select_one types_contrat</t>
+          <t>select_one situations</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>type_contrat</t>
+          <t>situation</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Type de contrat</t>
+          <t>Quelle est votre situation aujourd'hui ?</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1102,11 +1099,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>selected(${situation}, 'emploi')</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -1116,17 +1109,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>select_one types_activite</t>
+          <t>select_one types_contrat</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>type_activite</t>
+          <t>type_contrat</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Type d'activité exercée</t>
+          <t>Type de contrat</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1137,7 +1130,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>selected(${situation}, 'auto_emploi')</t>
+          <t>selected(${situation}, 'emploi')</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1149,17 +1142,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>select_one secteurs</t>
+          <t>select_one types_activite</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>secteur</t>
+          <t>type_activite</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Secteur d'activité</t>
+          <t>Type d'activité exercée</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1170,7 +1163,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>selected(${situation}, 'emploi') or selected(${situation}, 'auto_emploi') or selected(${situation}, 'stage')</t>
+          <t>selected(${situation}, 'auto_emploi')</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1182,17 +1175,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one secteurs</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>date_debut_activite</t>
+          <t>secteur</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Date de début de l'activité</t>
+          <t>Secteur d'activité</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1206,16 +1199,8 @@
           <t>selected(${situation}, 'emploi') or selected(${situation}, 'auto_emploi') or selected(${situation}, 'stage')</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>La date de début ne peut pas être dans le futur.</t>
-        </is>
-      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
@@ -1223,28 +1208,40 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>select_one tranches_revenu</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>revenu_tranche</t>
+          <t>date_debut_activite</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tranche de revenu mensuel</t>
+          <t>Date de début de l'activité</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>selected(${situation}, 'emploi') or selected(${situation}, 'auto_emploi')</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+          <t>selected(${situation}, 'emploi') or selected(${situation}, 'auto_emploi') or selected(${situation}, 'stage')</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>. &lt;= today()</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>La date de début ne peut pas être dans le futur.</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -1252,28 +1249,24 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>select_one liens_formation</t>
+          <t>select_one tranches_revenu</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>lien_formation</t>
+          <t>revenu_tranche</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Lien entre l'activité et la formation suivie</t>
+          <t>Tranche de revenu mensuel</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>selected(${situation}, 'emploi') or selected(${situation}, 'auto_emploi') or selected(${situation}, 'stage')</t>
+          <t>selected(${situation}, 'emploi') or selected(${situation}, 'auto_emploi')</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -1285,17 +1278,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one liens_formation</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>duree_recherche_mois</t>
+          <t>lien_formation</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Depuis combien de mois êtes-vous en recherche ?</t>
+          <t>Lien entre l'activité et la formation suivie</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1306,7 +1299,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>selected(${situation}, 'recherche')</t>
+          <t>selected(${situation}, 'emploi') or selected(${situation}, 'auto_emploi') or selected(${situation}, 'stage')</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -1318,24 +1311,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>select_multiple demarches</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>demarches</t>
+          <t>structure_accueil</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Démarches entreprises</t>
+          <t>Structure d'accueil du stage</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>selected(${situation}, 'recherche')</t>
+          <t>selected(${situation}, 'stage')</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1352,17 +1349,21 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>obstacle</t>
+          <t>nom_encadrant</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Principal obstacle rencontré</t>
+          <t>Nom de l'encadrant / maître de stage</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>selected(${situation}, 'stage')</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
@@ -1372,18 +1373,26 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>module_suivi</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>date_fin_stage</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Date de fin de stage prévue</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>selected(${situation}, 'stage')</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
@@ -1393,24 +1402,28 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>bascule</t>
+          <t>duree_recherche_mois</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Module 2 – Satisfaction</t>
+          <t>Depuis combien de mois êtes-vous en recherche ?</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>selected(${issue_contact}, 'joint')</t>
+          <t>selected(${situation}, 'recherche')</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -1422,26 +1435,26 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>select_one oui_non</t>
+          <t>select_multiple demarches</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>faire_satisfaction</t>
+          <t>demarches</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Réaliser le module satisfaction lors de ce contact ?</t>
+          <t>Démarches entreprises</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>selected(${situation}, 'recherche')</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
@@ -1451,30 +1464,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>select_one cycles</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>obstacle</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cycle d'enquête</t>
+          <t>Principal obstacle rencontré</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
@@ -1489,21 +1494,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>consigne_notes</t>
+          <t>consigne_profil</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sur une échelle de 1 à 5, où 1 signifie « pas du tout satisfait » et 5 « très satisfait », comment évaluez-vous les éléments suivants ?</t>
+          <t>Les deux questions suivantes mettent à jour la fiche du bénéficiaire (utile si ce n'était pas connu à l'inscription) - répondez-y seulement si vous avez l'information.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
@@ -1513,30 +1514,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>select_one echelle_5</t>
+          <t>select_one oui_non</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>note_formation</t>
+          <t>refugie</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>La formation dans son ensemble</t>
+          <t>Le/la bénéficiaire est-il/elle réfugié(e) ?</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
@@ -1546,17 +1539,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>select_one echelle_5</t>
+          <t>select_one pays_origine</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>note_formateurs</t>
+          <t>pays_origine</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Les formateurs</t>
+          <t>Pays d'origine</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1567,7 +1560,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
+          <t>selected(${refugie}, 'oui')</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -1579,30 +1572,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>select_one echelle_5</t>
+          <t>select_one oui_non</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>note_contenus</t>
+          <t>handicap</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Les contenus pédagogiques</t>
+          <t>Le/la bénéficiaire est-il/elle en situation de handicap ?</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
@@ -1612,17 +1597,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>select_one echelle_5</t>
+          <t>select_one type_handicap</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>note_equipements</t>
+          <t>type_handicap</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Les équipements et le matériel</t>
+          <t>Type de handicap</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1633,7 +1618,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
+          <t>selected(${handicap}, 'oui')</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -1645,30 +1630,18 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>select_one echelle_5</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>note_conditions</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Les conditions d'accueil</t>
-        </is>
-      </c>
+          <t>module_suivi</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
@@ -1678,28 +1651,24 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>select_one amelioration</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>employabilite</t>
+          <t>bascule</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>La formation a-t-elle amélioré votre employabilité ?</t>
+          <t>Module 2 – Satisfaction</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
+          <t>selected(${issue_contact}, 'joint')</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -1716,12 +1685,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>recommande</t>
+          <t>faire_satisfaction</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Recommanderiez-vous la formation à une autre personne ?</t>
+          <t>Réaliser le module satisfaction lors de ce contact ?</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1730,11 +1699,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>selected(${faire_satisfaction}, 'oui')</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
@@ -1744,24 +1709,28 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one cycles</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>raison_non</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Pour quelle raison ?</t>
+          <t>Cycle d'enquête</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>selected(${recommande}, 'non')</t>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -1773,17 +1742,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>point_fort</t>
+          <t>consigne_notes</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Qu'est-ce qui a le mieux fonctionné ?</t>
+          <t>Sur une échelle de 1 à 5, où 1 signifie « pas du tout satisfait » et 5 « très satisfait », comment évaluez-vous les éléments suivants ?</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1802,21 +1771,25 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one echelle_5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>point_amelioration</t>
+          <t>note_formation</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Qu'est-ce qu'il faudrait améliorer ?</t>
+          <t>La formation dans son ensemble</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>selected(${faire_satisfaction}, 'oui')</t>
@@ -1831,18 +1804,30 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>select_one echelle_5</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>bascule</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>note_formateurs</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Les formateurs</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
@@ -1852,27 +1837,300 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one echelle_5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>observations</t>
+          <t>note_contenus</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Observations de l'enquêteur</t>
+          <t>Les contenus pédagogiques</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>select_one echelle_5</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>note_equipements</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Les équipements et le matériel</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>select_one echelle_5</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>note_conditions</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Les conditions d'accueil</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>select_one amelioration</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>employabilite</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>La formation a-t-elle amélioré votre employabilité ?</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>recommande</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Recommanderiez-vous la formation à une autre personne ?</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>raison_non</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Pour quelle raison ?</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>selected(${recommande}, 'non')</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>point_fort</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Qu'est-ce qui a le mieux fonctionné ?</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>point_amelioration</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Qu'est-ce qu'il faudrait améliorer ?</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>selected(${faire_satisfaction}, 'oui')</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>bascule</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>observations</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Observations de l'enquêteur</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1885,7 +2143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2946,6 +3204,176 @@
       <c r="C63" t="inlineStr">
         <is>
           <t>Pas du tout</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>pays_origine</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>somalie</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Somalie</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>pays_origine</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ethiopie</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Éthiopie</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>pays_origine</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>yemen</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Yémen</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>pays_origine</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>erythree</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Érythrée</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>pays_origine</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>autre</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Autre</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>type_handicap</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>moteur</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Moteur</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>type_handicap</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>visuel</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Visuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>type_handicap</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>auditif</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Auditif</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>type_handicap</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>intellectuel</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Intellectuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>type_handicap</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>autre</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Autre</t>
         </is>
       </c>
     </row>

</xml_diff>